<commit_message>
refactor(daq): data-driven telegraf config & query alignment
</commit_message>
<xml_diff>
--- a/src_matlab/stream_test/telegraf_settings.xlsx
+++ b/src_matlab/stream_test/telegraf_settings.xlsx
@@ -5,16 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeehyun/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeehyun/Desktop/optical-gvt-daq/src_matlab/stream_test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{791A7F0C-876D-FA4E-8F10-0D0B95398443}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B844F79-36D0-B148-98D3-E86943578D69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19880" xr2:uid="{74B92C5B-7F41-7F4D-9F5D-9CE4AA5ECC7F}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19840" activeTab="2" xr2:uid="{74B92C5B-7F41-7F4D-9F5D-9CE4AA5ECC7F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="35">
   <si>
     <t>Telegraf_IP</t>
   </si>
@@ -78,9 +79,6 @@
     <t>Network_Settings</t>
   </si>
   <si>
-    <t>Parameter</t>
-  </si>
-  <si>
     <t>Value</t>
   </si>
   <si>
@@ -103,13 +101,58 @@
   </si>
   <si>
     <t>Experimental_Matrix</t>
+  </si>
+  <si>
+    <t>Key</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Assignment</t>
+  </si>
+  <si>
+    <t>packet_counter</t>
+  </si>
+  <si>
+    <t>uint32</t>
+  </si>
+  <si>
+    <t>field</t>
+  </si>
+  <si>
+    <t>velocity</t>
+  </si>
+  <si>
+    <t>float32</t>
+  </si>
+  <si>
+    <t>alpha</t>
+  </si>
+  <si>
+    <t>lift</t>
+  </si>
+  <si>
+    <t>run_id</t>
+  </si>
+  <si>
+    <t>test_point</t>
+  </si>
+  <si>
+    <t>string</t>
+  </si>
+  <si>
+    <t>tag</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -164,6 +207,19 @@
       <name val="Helvetica Neue"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -201,7 +257,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -227,6 +283,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -254,10 +316,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -585,20 +643,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.2">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
+      <c r="B1" s="13"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
     </row>
     <row r="2" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>13</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="9"/>
@@ -663,15 +721,15 @@
     </row>
     <row r="9" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>14</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B10" s="3">
         <v>2</v>
@@ -698,21 +756,21 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A1" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
+      <c r="A1" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
     </row>
     <row r="2" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="7" t="s">
         <v>18</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.2">
@@ -754,4 +812,96 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3628DD43-0D43-1F4B-ACFF-1A50150DFBFD}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A1" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A2" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A3" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A4" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A5" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A6" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="18" x14ac:dyDescent="0.2">
+      <c r="A7" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>